<commit_message>
Update all 4 routine files with latest author versions (password 677527315)
https://claude.ai/code/session_013goGtNxneCGLBYieXpHUZd
</commit_message>
<xml_diff>
--- a/assets/rutinas-hombre-simple-progresion.xlsx
+++ b/assets/rutinas-hombre-simple-progresion.xlsx
@@ -36,7 +36,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="28">
     <font>
       <name val="Arial"/>
       <charset val="1"/>
@@ -202,8 +202,39 @@
       <color rgb="FF3A3A3A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FFD9D9D9"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF7CB518"/>
+      <sz val="13"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF7CB518"/>
+      <sz val="12"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="FF8A938C"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -316,6 +347,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF0EAF2"/>
         <bgColor rgb="FFF5F0E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B0F0D"/>
+        <bgColor rgb="FF0B0F0D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7CB518"/>
+        <bgColor rgb="FF7CB518"/>
       </patternFill>
     </fill>
   </fills>
@@ -458,7 +501,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="218">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1112,6 +1155,23 @@
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1458,15 +1518,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="J11:P25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="94" min="1" max="1"/>
+    <col width="1.5" customWidth="1" style="94" min="10" max="10"/>
+    <col width="11" customWidth="1" style="94" min="11" max="11"/>
+    <col width="11" customWidth="1" style="94" min="12" max="12"/>
+    <col width="11" customWidth="1" style="94" min="13" max="13"/>
+    <col width="11" customWidth="1" style="94" min="14" max="14"/>
+    <col width="11" customWidth="1" style="94" min="15" max="15"/>
+    <col width="1.5" customWidth="1" style="94" min="16" max="16"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="11" ht="4.5" customHeight="1" s="94">
+      <c r="J11" s="211" t="n"/>
+      <c r="K11" s="211" t="n"/>
+      <c r="L11" s="211" t="n"/>
+      <c r="M11" s="211" t="n"/>
+      <c r="N11" s="211" t="n"/>
+      <c r="O11" s="211" t="n"/>
+      <c r="P11" s="211" t="n"/>
+    </row>
+    <row r="12" ht="10" customHeight="1" s="94">
+      <c r="J12" s="212" t="n"/>
+      <c r="K12" s="212" t="n"/>
+      <c r="L12" s="212" t="n"/>
+      <c r="M12" s="212" t="n"/>
+      <c r="N12" s="212" t="n"/>
+      <c r="O12" s="212" t="n"/>
+      <c r="P12" s="212" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="94">
+      <c r="J13" s="212" t="n"/>
+      <c r="K13" s="213" t="inlineStr">
+        <is>
+          <t>¿Te han resultado útiles estas rutinas?</t>
+        </is>
+      </c>
+      <c r="P13" s="212" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1" s="94">
+      <c r="J14" s="212" t="n"/>
+      <c r="P14" s="212" t="n"/>
+    </row>
+    <row r="15" ht="16" customHeight="1" s="94">
+      <c r="J15" s="212" t="n"/>
+      <c r="K15" s="214" t="inlineStr">
+        <is>
+          <t>Entonces hay más esperándote: en mi web y en Instagram comparto consejos prácticos —sin humo— para entrenar con cabeza, comer bien y construir una salud que dure años.</t>
+        </is>
+      </c>
+      <c r="P15" s="212" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" s="94">
+      <c r="J16" s="212" t="n"/>
+      <c r="P16" s="212" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1" s="94">
+      <c r="J17" s="212" t="n"/>
+      <c r="P17" s="212" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1" s="94">
+      <c r="J18" s="212" t="n"/>
+      <c r="P18" s="212" t="n"/>
+    </row>
+    <row r="19" ht="10" customHeight="1" s="94">
+      <c r="J19" s="212" t="n"/>
+      <c r="K19" s="212" t="n"/>
+      <c r="L19" s="212" t="n"/>
+      <c r="M19" s="212" t="n"/>
+      <c r="N19" s="212" t="n"/>
+      <c r="O19" s="212" t="n"/>
+      <c r="P19" s="212" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1" s="94">
+      <c r="J20" s="212" t="n"/>
+      <c r="K20" s="215" t="inlineStr">
+        <is>
+          <t>www.rubensoro.es</t>
+        </is>
+      </c>
+      <c r="P20" s="212" t="n"/>
+    </row>
+    <row r="21" ht="6" customHeight="1" s="94">
+      <c r="J21" s="212" t="n"/>
+      <c r="K21" s="212" t="n"/>
+      <c r="L21" s="212" t="n"/>
+      <c r="M21" s="212" t="n"/>
+      <c r="N21" s="212" t="n"/>
+      <c r="O21" s="212" t="n"/>
+      <c r="P21" s="212" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1" s="94">
+      <c r="J22" s="212" t="n"/>
+      <c r="K22" s="216" t="inlineStr">
+        <is>
+          <t>Instagram · @rubensoro.seduenodetucuerpo</t>
+        </is>
+      </c>
+      <c r="P22" s="212" t="n"/>
+    </row>
+    <row r="23" ht="10" customHeight="1" s="94">
+      <c r="J23" s="212" t="n"/>
+      <c r="K23" s="212" t="n"/>
+      <c r="L23" s="212" t="n"/>
+      <c r="M23" s="212" t="n"/>
+      <c r="N23" s="212" t="n"/>
+      <c r="O23" s="212" t="n"/>
+      <c r="P23" s="212" t="n"/>
+    </row>
+    <row r="24" ht="16" customHeight="1" s="94">
+      <c r="J24" s="212" t="n"/>
+      <c r="K24" s="217" t="inlineStr">
+        <is>
+          <t>Nos vemos dentro. — Rubén</t>
+        </is>
+      </c>
+      <c r="P24" s="212" t="n"/>
+    </row>
+    <row r="25" ht="10" customHeight="1" s="94">
+      <c r="J25" s="212" t="n"/>
+      <c r="K25" s="212" t="n"/>
+      <c r="L25" s="212" t="n"/>
+      <c r="M25" s="212" t="n"/>
+      <c r="N25" s="212" t="n"/>
+      <c r="O25" s="212" t="n"/>
+      <c r="P25" s="212" t="n"/>
+    </row>
+  </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="851A"/>
+  <mergeCells count="5">
+    <mergeCell ref="K20:O20"/>
+    <mergeCell ref="K13:O14"/>
+    <mergeCell ref="K24:O24"/>
+    <mergeCell ref="K15:O18"/>
+    <mergeCell ref="K22:O22"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>